<commit_message>
Add stock poster images and styles
</commit_message>
<xml_diff>
--- a/Poster Collection.xlsx
+++ b/Poster Collection.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1601" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1671" uniqueCount="353">
   <si>
     <t>Date</t>
   </si>
@@ -500,6 +500,9 @@
     <t>Expressobeans Poster Link</t>
   </si>
   <si>
+    <t>Stock Image</t>
+  </si>
+  <si>
     <t>Gary Baseman</t>
   </si>
   <si>
@@ -509,24 +512,36 @@
     <t>https://expressobeans.com/public/detail.php/123494</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1vLdapZu2Oj-jWqdahQWtxtTh6grXWBK6/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Gerald Scarfe</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/151915</t>
   </si>
   <si>
-    <t>Kii Arens</t>
+    <t>https://drive.google.com/file/d/1WHemrT9ldrXhN-D_Ddouo92zj4kF7swm/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>Rob Sheridan, Russell Mills</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/179172</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/15JpqRB4rJhrhJrA67Kk8mu6RidC1UBRA/view?usp=drive_link</t>
+  </si>
+  <si>
     <t xml:space="preserve">Arens, Kii, Plastic Jesus </t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/186961</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1xuLmHvGKSXCHMIoQ0Qei1UGtdZ5O_TEj/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Brad Klausen</t>
   </si>
   <si>
@@ -536,18 +551,27 @@
     <t>https://expressobeans.com/public/detail.php/194219</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1Cdr6HCwHruHIvXDnshMWKLxGb07QuRnk/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Ames Brothers</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/194934</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1_oSRhhUR8OqSshawfmYXLAim5Y6mrY2v/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Rob Jones</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/196278</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1ytGWzHsqf1bMSDgZQ6EdKPkTP7yUZK02/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Sket One</t>
   </si>
   <si>
@@ -560,6 +584,9 @@
     <t>https://expressobeans.com/public/detail.php/208452</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1fFctIb_RYxTDxFhpjmRfX3N5MCyJTUs0/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Todd Slater</t>
   </si>
   <si>
@@ -569,39 +596,60 @@
     <t>https://expressobeans.com/public/detail.php/211539</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1wSPyeKU5t347PxeDocOEEpUf2FiRU94R/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Jared Connor</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/212319</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1ruJQUS42sO_n4WtttnHkIg90wic236iH/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Pale Horse</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/218675</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1CqmCXx4HVZFyi98cYws081u3fTw5-ifw/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Adi Granov</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/222040</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1sHsEgQd5SEVy0ngM7jzkQzTXS2MqGhye/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Gregg Gordon</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/225691</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1Y-Rpnb-BhEi6cnj8J-uJogItdZFhIAUv/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>https://expressobeans.com/public/detail.php/240144</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1PfmnWHFKHA7TM8jfN1qCFZu8CgT336J2/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Adam Jones</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/290999</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/10huhLiaF_EBaakEdrYtrVzj_yuwA0Dso/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Unknown</t>
   </si>
   <si>
@@ -617,12 +665,18 @@
     <t>https://expressobeans.com/public/detail.php/244301</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1AFKuZc-0h-a6uiglL4r-vTAZoB3GYe3q/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Angryblue (Justin Kamerer)</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/253928</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1MJPtKpbN45L5b8EpBhMFl-s3789-61Z4/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Emek</t>
   </si>
   <si>
@@ -632,30 +686,54 @@
     <t>https://expressobeans.com/public/detail.php/247251</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1tLUsltydRdYEiv3OVKAUo0bcdzsNMbC2/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1kPWEuHbBVO5WY0bVVtJmgsYnXOdbMmnf/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>https://expressobeans.com/public/detail.php/281506</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1PPm8DH6HuJc3qBh95sAEMEBWcD5kEjiw/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Ian Williams</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/265755</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1TZUjbOZ_7HrEDyJ_1v2nGCOYtYgN4dd_/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Jamie Koala</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/323469</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1ibuMP3F31TlkCcjDhlvYIBcrpgBf2keG/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ybLG2V639yGEIcgELiSucG-yuBQ-EdfP/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>https://expressobeans.com/public/detail.php/274618</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1uJjbTBnu3vgkQgB_YDUOIfsLBwRsz9zl/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Erica Williams</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/273538</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1cn8nnnrlL9PkWDtAgC7uucUu3dTCOYaq/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Hatch Show Print</t>
   </si>
   <si>
@@ -665,18 +743,30 @@
     <t>https://expressobeans.com/public/detail.php/306265</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1GroJCI6_OBNmhVnTqDncCUxnzMuHwyuN/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Arian Buhler</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1ZcoDdTTyDQQRnSoGEHZSjDaQRhlPDjAr/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>https://expressobeans.com/public/detail.php/280905</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/12moXxf74fYWjuf1YwoBGsqk01ZPicn0k/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Allen Williams</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/280401</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1UZFdLC1G8ylHU4sEAp9hDnHJs-4V3cPf/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Chet Zar</t>
   </si>
   <si>
@@ -686,183 +776,291 @@
     <t>https://expressobeans.com/public/detail.php/280931</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1v2LsCmM9fvl_W3gFnQR1q11_4Q3bVS32/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Dominic Hailstone</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/280944</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1h0-gV-COgeHT2trdlb5i_LeEzbob2Twj/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Landland</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/306381</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1hOUd3Ho8E8iMix8Dartijjph-2xK_2zv/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Robert Banach</t>
   </si>
   <si>
-    <t>Angryblue</t>
+    <t>https://drive.google.com/file/d/1kkLJ28wGH1QLr1Mhv0Fn_aqW_AsXts0z/view?usp=drive_link</t>
   </si>
   <si>
     <t>Official / TBD</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1ThrtMznodlRzPz4TmMpZWiu4VJMVVczV/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>https://expressobeans.com/public/detail.php/302663</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/10aeSKg2MIn5nFuMERoEYVHpvs59nagtC/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Frank Frazetta</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/303923</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1fQ1sE7GsXJt5ygB_s_zhKMdHUN6ExaHQ/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Alex Grey</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/304419</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/14HljZ2q6ElxzwE4Hm0NAIpnVUBOyStET/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>John Crawford</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/319934</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1HxIRaudrAUcywZePbxbVi_S6D7Sxa521/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Michael Hacker</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/306690</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1htrKPNVj-S0rzMDKVHaDxXbavqFV7r-R/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Virgil Abloh / Official</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/307864</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1IaMV1J12N4wARQE3GhHl4F1JbjDClc2_/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Official / Zoran Bihac (Creative Dir)</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/309873</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1YKlNPfvCOIDbwIV2qWq627nBLtYyME6m/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>https://expressobeans.com/public/detail.php/309569</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/13LX2SWcSuzT7_LA8EqPttebbhNVVIhU8/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/11oBTGgWQYNDDksZWyi-0gVYj1MHQ7r-0/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Alex Kuno</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/314300</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/16fjtNAhMmh7uSzxS3s_SBquUFb2e_Gwm/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Squindo</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/316748</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1JS85U6pJgzgzHWbnnpEA1cZm1-EWHtki/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>https://expressobeans.com/public/detail.php/316749</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/11rXvBpw_IEvRafv7j6rcaAGOQFMEhkUC/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Studio/Official</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/318464</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/16Fx-YdHD426RyHt8cDAkEsENznw1pTOl/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Travis Gillan</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/318753</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1fgrwQihWRHbUsj7phoWI3lnKoEc03CRQ/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Miles Johnston</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/323237</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1KEydOB85Nhf8o6zV5j2q3wE3-oaPRV2W/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Richard Biffle</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/317772</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1pgCttfdwE6PwjzaH6qunpp7G6zAaCCow/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Liz Passerieux</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/321059</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1B1ZRIn_c32uVblQk97RAft4zB-XkYcy6/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Sty8eQ06_Xbqos0F4MdU4W_i7NlC8ZEB/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Korin Faught</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/321675</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/14znodZhEdb_9jUMVy6sDkm86lnKXcQjH/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Zoltron</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/322555</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/17pqvG9lxO-l0Vdtn75W3BHycXa83q5wL/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Zeb Love</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/322934</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1Qkpq7hT7UIqar7whgNWj_qigUOHFoe-R/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Mark Dean Veca</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/322926</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/13KIgofdy7hwVwK_6fqCTQOGHMEyZQVXk/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Logan Schmitt</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1qJxf2GjitO6wOgkHzzwx-Q98aBYH4b7w/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Burrito Breath</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/324915</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1dQOUEbXdmdukUbg1XXcAN6VNQS4gdDTJ/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1kyyIotG2C77JYkdTB4Syp89Sz7uRr31q/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>DABSMYLA</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/331952</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1nhnWVdsZGFIYWxQGq15GNVykvmGD7HzK/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Don Pendleton</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/332084</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1gg5tC0lsj8zRQwzL5Q0-B5KJBMIjwmAC/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Miles Tsang</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/332464</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1THs_y6kRcVTGqyDzchULz_i9ZYh4FPgH/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>NC Winters</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/332529</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/17obLPftp_3RHHG5aOhpIzfHetQ0UWplM/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1awJQBEATeuaBSgz4H96upvKVQruDakRX/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Peel it back</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/334688</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1Y4fr0EWZpdKN7RAhC7iOQt28ajYHQ6Hs/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>Boop a Doop</t>
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/339059</t>
   </si>
   <si>
+    <t>https://drive.google.com/file/d/1EnNoXeBEvJKLqF6oI9aqfkhm0VS9z5d7/view?usp=drive_link</t>
+  </si>
+  <si>
     <t>AVVT/PTTN</t>
   </si>
   <si>
@@ -873,6 +1071,9 @@
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/339352</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1t0V2HQrDpkYGYF8XyljYkxtAdmIzeFDj/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
@@ -4090,6 +4291,9 @@
       <c r="O1" s="1" t="s">
         <v>160</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7">
@@ -4099,7 +4303,7 @@
         <v>140</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>123</v>
@@ -4108,7 +4312,7 @@
         <v>81</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>143</v>
@@ -4132,7 +4336,10 @@
         <v>10</v>
       </c>
       <c r="O2" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="3">
@@ -4143,7 +4350,7 @@
         <v>105</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>106</v>
@@ -4174,7 +4381,10 @@
         <v>10</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="4">
@@ -4185,7 +4395,7 @@
         <v>58</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>14</v>
@@ -4216,7 +4426,10 @@
         <v>10</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="5">
@@ -4227,7 +4440,7 @@
         <v>80</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>14</v>
@@ -4258,7 +4471,10 @@
         <v>10</v>
       </c>
       <c r="O5" s="8" t="s">
-        <v>169</v>
+        <v>173</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="6">
@@ -4269,7 +4485,7 @@
         <v>80</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>100</v>
@@ -4294,7 +4510,7 @@
         <v>19</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="M6" s="1" t="s">
         <v>104</v>
@@ -4303,7 +4519,10 @@
         <v>10</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>172</v>
+        <v>177</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="7">
@@ -4314,7 +4533,7 @@
         <v>136</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>137</v>
@@ -4345,7 +4564,10 @@
         <v>10</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>174</v>
+        <v>180</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="8">
@@ -4356,7 +4578,7 @@
         <v>112</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>106</v>
@@ -4387,7 +4609,10 @@
         <v>10</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>176</v>
+        <v>183</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="9">
@@ -4398,7 +4623,7 @@
         <v>140</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>106</v>
@@ -4407,7 +4632,7 @@
         <v>81</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>141</v>
@@ -4425,7 +4650,7 @@
         <v>19</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="M9" s="1" t="s">
         <v>104</v>
@@ -4434,7 +4659,10 @@
         <v>10</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>180</v>
+        <v>188</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="10">
@@ -4445,7 +4673,7 @@
         <v>113</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>106</v>
@@ -4454,7 +4682,7 @@
         <v>35</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>114</v>
@@ -4478,7 +4706,10 @@
         <v>10</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>183</v>
+        <v>192</v>
+      </c>
+      <c r="P10" s="3" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="11">
@@ -4489,7 +4720,7 @@
         <v>140</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>14</v>
@@ -4520,7 +4751,10 @@
         <v>10</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>185</v>
+        <v>195</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="12">
@@ -4531,7 +4765,7 @@
         <v>41</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>38</v>
@@ -4565,7 +4799,10 @@
         <v>10</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>187</v>
+        <v>198</v>
+      </c>
+      <c r="P12" s="3" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="13">
@@ -4576,7 +4813,7 @@
         <v>54</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>38</v>
@@ -4607,7 +4844,10 @@
         <v>10</v>
       </c>
       <c r="O13" s="8" t="s">
-        <v>189</v>
+        <v>201</v>
+      </c>
+      <c r="P13" s="3" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="14">
@@ -4618,7 +4858,7 @@
         <v>41</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>14</v>
@@ -4649,7 +4889,10 @@
         <v>10</v>
       </c>
       <c r="O14" s="8" t="s">
-        <v>191</v>
+        <v>204</v>
+      </c>
+      <c r="P14" s="3" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="15">
@@ -4660,7 +4903,7 @@
         <v>37</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>106</v>
@@ -4691,7 +4934,10 @@
         <v>10</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>192</v>
+        <v>206</v>
+      </c>
+      <c r="P15" s="3" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="16">
@@ -4702,7 +4948,7 @@
         <v>54</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>64</v>
@@ -4736,7 +4982,10 @@
         <v>10</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>194</v>
+        <v>209</v>
+      </c>
+      <c r="P16" s="3" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="17">
@@ -4747,7 +4996,7 @@
         <v>54</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>64</v>
@@ -4757,7 +5006,7 @@
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="9" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>17</v>
@@ -4772,11 +5021,14 @@
         <v>19</v>
       </c>
       <c r="L17" s="9" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="N17" s="10"/>
       <c r="O17" s="3" t="s">
-        <v>194</v>
+        <v>209</v>
+      </c>
+      <c r="P17" s="3" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="18">
@@ -4784,10 +5036,10 @@
         <v>42958.0</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>72</v>
@@ -4821,7 +5073,10 @@
         <v>10</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>199</v>
+        <v>215</v>
+      </c>
+      <c r="P18" s="3" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="19">
@@ -4832,7 +5087,7 @@
         <v>105</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>106</v>
@@ -4863,7 +5118,10 @@
         <v>10</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>201</v>
+        <v>218</v>
+      </c>
+      <c r="P19" s="3" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="20">
@@ -4874,10 +5132,10 @@
         <v>80</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>202</v>
+        <v>220</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>203</v>
+        <v>221</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>35</v>
@@ -4905,7 +5163,10 @@
         <v>10</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>204</v>
+        <v>222</v>
+      </c>
+      <c r="P20" s="3" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="21">
@@ -4916,7 +5177,7 @@
         <v>132</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>32</v>
@@ -4946,6 +5207,9 @@
       <c r="N21" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="P21" s="8" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7">
@@ -4955,7 +5219,7 @@
         <v>54</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>32</v>
@@ -4986,7 +5250,10 @@
         <v>10</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>205</v>
+        <v>225</v>
+      </c>
+      <c r="P22" s="8" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="23">
@@ -4997,7 +5264,7 @@
         <v>91</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>206</v>
+        <v>227</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>106</v>
@@ -5028,7 +5295,10 @@
         <v>10</v>
       </c>
       <c r="O23" s="8" t="s">
-        <v>207</v>
+        <v>228</v>
+      </c>
+      <c r="P23" s="8" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="24">
@@ -5039,7 +5309,7 @@
         <v>118</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>208</v>
+        <v>230</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>38</v>
@@ -5073,7 +5343,10 @@
         <v>10</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>209</v>
+        <v>231</v>
+      </c>
+      <c r="P24" s="8" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="25">
@@ -5111,6 +5384,9 @@
       <c r="N25" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="P25" s="8" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7">
@@ -5120,7 +5396,7 @@
         <v>37</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>14</v>
@@ -5151,7 +5427,10 @@
         <v>10</v>
       </c>
       <c r="O26" s="8" t="s">
-        <v>210</v>
+        <v>234</v>
+      </c>
+      <c r="P26" s="8" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="27">
@@ -5162,7 +5441,7 @@
         <v>37</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>211</v>
+        <v>236</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>14</v>
@@ -5193,7 +5472,10 @@
         <v>10</v>
       </c>
       <c r="O27" s="3" t="s">
-        <v>212</v>
+        <v>237</v>
+      </c>
+      <c r="P27" s="8" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="28">
@@ -5204,7 +5486,7 @@
         <v>87</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>213</v>
+        <v>239</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>14</v>
@@ -5243,7 +5525,7 @@
         <v>133</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>214</v>
+        <v>240</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>134</v>
@@ -5274,7 +5556,10 @@
         <v>10</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>215</v>
+        <v>241</v>
+      </c>
+      <c r="P29" s="8" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="30">
@@ -5282,10 +5567,10 @@
         <v>43733.0</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>216</v>
+        <v>243</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>38</v>
@@ -5318,6 +5603,9 @@
       <c r="N30" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="P30" s="8" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7">
@@ -5327,7 +5615,7 @@
         <v>54</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>123</v>
@@ -5361,7 +5649,10 @@
         <v>10</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>217</v>
+        <v>245</v>
+      </c>
+      <c r="P31" s="8" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="32">
@@ -5372,7 +5663,7 @@
         <v>54</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>218</v>
+        <v>247</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>14</v>
@@ -5406,7 +5697,10 @@
         <v>10</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>219</v>
+        <v>248</v>
+      </c>
+      <c r="P32" s="8" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="33">
@@ -5417,7 +5711,7 @@
         <v>54</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>126</v>
@@ -5442,7 +5736,7 @@
         <v>18</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>221</v>
+        <v>251</v>
       </c>
       <c r="M33" s="1" t="s">
         <v>104</v>
@@ -5451,7 +5745,10 @@
         <v>10</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>222</v>
+        <v>252</v>
+      </c>
+      <c r="P33" s="8" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="34">
@@ -5462,7 +5759,7 @@
         <v>54</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>223</v>
+        <v>254</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>29</v>
@@ -5493,7 +5790,10 @@
         <v>10</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>224</v>
+        <v>255</v>
+      </c>
+      <c r="P34" s="8" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="35">
@@ -5504,7 +5804,7 @@
         <v>87</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>213</v>
+        <v>239</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>88</v>
@@ -5546,7 +5846,7 @@
         <v>62</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>225</v>
+        <v>257</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>14</v>
@@ -5577,7 +5877,10 @@
         <v>10</v>
       </c>
       <c r="O36" s="8" t="s">
-        <v>226</v>
+        <v>258</v>
+      </c>
+      <c r="P36" s="8" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="37">
@@ -5585,10 +5888,10 @@
         <v>44468.0</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>227</v>
+        <v>260</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>14</v>
@@ -5618,6 +5921,9 @@
       <c r="N37" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="P37" s="3" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7">
@@ -5627,7 +5933,7 @@
         <v>51</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>228</v>
+        <v>262</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>52</v>
@@ -5658,6 +5964,9 @@
       </c>
       <c r="N38" s="3" t="s">
         <v>10</v>
+      </c>
+      <c r="P38" s="8" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="39">
@@ -5668,7 +5977,7 @@
         <v>84</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>229</v>
+        <v>262</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>14</v>
@@ -5699,7 +6008,10 @@
         <v>10</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>230</v>
+        <v>264</v>
+      </c>
+      <c r="P39" s="8" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="40">
@@ -5710,7 +6022,7 @@
         <v>54</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>231</v>
+        <v>266</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>128</v>
@@ -5744,7 +6056,10 @@
         <v>10</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>232</v>
+        <v>267</v>
+      </c>
+      <c r="P40" s="3" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="41">
@@ -5755,7 +6070,7 @@
         <v>54</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>233</v>
+        <v>269</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>131</v>
@@ -5786,7 +6101,10 @@
         <v>10</v>
       </c>
       <c r="O41" s="8" t="s">
-        <v>234</v>
+        <v>270</v>
+      </c>
+      <c r="P41" s="3" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="42">
@@ -5797,7 +6115,7 @@
         <v>58</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>235</v>
+        <v>272</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>14</v>
@@ -5828,7 +6146,10 @@
         <v>10</v>
       </c>
       <c r="O42" s="8" t="s">
-        <v>236</v>
+        <v>273</v>
+      </c>
+      <c r="P42" s="3" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="43">
@@ -5839,7 +6160,7 @@
         <v>58</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>235</v>
+        <v>272</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>14</v>
@@ -5870,7 +6191,10 @@
         <v>10</v>
       </c>
       <c r="O43" s="8" t="s">
-        <v>236</v>
+        <v>273</v>
+      </c>
+      <c r="P43" s="3" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="44">
@@ -5881,7 +6205,7 @@
         <v>41</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>237</v>
+        <v>275</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>43</v>
@@ -5914,7 +6238,10 @@
         <v>10</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>238</v>
+        <v>276</v>
+      </c>
+      <c r="P44" s="3" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="45">
@@ -5925,7 +6252,7 @@
         <v>76</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>239</v>
+        <v>278</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>14</v>
@@ -5956,7 +6283,10 @@
         <v>10</v>
       </c>
       <c r="O45" s="3" t="s">
-        <v>240</v>
+        <v>279</v>
+      </c>
+      <c r="P45" s="3" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="46">
@@ -5967,7 +6297,7 @@
         <v>92</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>241</v>
+        <v>281</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>93</v>
@@ -5998,7 +6328,10 @@
         <v>10</v>
       </c>
       <c r="O46" s="3" t="s">
-        <v>242</v>
+        <v>282</v>
+      </c>
+      <c r="P46" s="3" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="47">
@@ -6009,7 +6342,7 @@
         <v>41</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>38</v>
@@ -6040,7 +6373,10 @@
         <v>10</v>
       </c>
       <c r="O47" s="3" t="s">
-        <v>243</v>
+        <v>284</v>
+      </c>
+      <c r="P47" s="3" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="48">
@@ -6051,7 +6387,7 @@
         <v>51</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>52</v>
@@ -6082,6 +6418,9 @@
       </c>
       <c r="N48" s="3" t="s">
         <v>10</v>
+      </c>
+      <c r="P48" s="8" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="49">
@@ -6092,7 +6431,7 @@
         <v>54</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>244</v>
+        <v>287</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>52</v>
@@ -6123,7 +6462,10 @@
         <v>10</v>
       </c>
       <c r="O49" s="3" t="s">
-        <v>245</v>
+        <v>288</v>
+      </c>
+      <c r="P49" s="8" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="50">
@@ -6134,7 +6476,7 @@
         <v>37</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>246</v>
+        <v>290</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>46</v>
@@ -6168,7 +6510,10 @@
         <v>10</v>
       </c>
       <c r="O50" s="8" t="s">
-        <v>247</v>
+        <v>291</v>
+      </c>
+      <c r="P50" s="8" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="51">
@@ -6179,7 +6524,7 @@
         <v>37</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>246</v>
+        <v>290</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>46</v>
@@ -6213,7 +6558,10 @@
         <v>10</v>
       </c>
       <c r="O51" s="3" t="s">
-        <v>248</v>
+        <v>293</v>
+      </c>
+      <c r="P51" s="3" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="52">
@@ -6224,7 +6572,7 @@
         <v>28</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>249</v>
+        <v>295</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>29</v>
@@ -6256,7 +6604,10 @@
         <v>10</v>
       </c>
       <c r="O52" s="3" t="s">
-        <v>250</v>
+        <v>296</v>
+      </c>
+      <c r="P52" s="3" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="53">
@@ -6267,7 +6618,7 @@
         <v>13</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>251</v>
+        <v>298</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>14</v>
@@ -6300,7 +6651,10 @@
         <v>10</v>
       </c>
       <c r="O53" s="3" t="s">
-        <v>252</v>
+        <v>299</v>
+      </c>
+      <c r="P53" s="3" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="54">
@@ -6311,7 +6665,7 @@
         <v>13</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>253</v>
+        <v>301</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>14</v>
@@ -6342,7 +6696,10 @@
         <v>10</v>
       </c>
       <c r="O54" s="8" t="s">
-        <v>254</v>
+        <v>302</v>
+      </c>
+      <c r="P54" s="3" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="55">
@@ -6353,7 +6710,7 @@
         <v>42</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>255</v>
+        <v>304</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>14</v>
@@ -6384,7 +6741,10 @@
         <v>10</v>
       </c>
       <c r="O55" s="8" t="s">
-        <v>256</v>
+        <v>305</v>
+      </c>
+      <c r="P55" s="8" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="56">
@@ -6395,7 +6755,7 @@
         <v>54</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>257</v>
+        <v>307</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>38</v>
@@ -6426,7 +6786,10 @@
         <v>10</v>
       </c>
       <c r="O56" s="3" t="s">
-        <v>258</v>
+        <v>308</v>
+      </c>
+      <c r="P56" s="8" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="57">
@@ -6437,7 +6800,7 @@
         <v>54</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>257</v>
+        <v>307</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>38</v>
@@ -6468,7 +6831,10 @@
         <v>10</v>
       </c>
       <c r="O57" s="3" t="s">
-        <v>258</v>
+        <v>308</v>
+      </c>
+      <c r="P57" s="8" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="58">
@@ -6479,7 +6845,7 @@
         <v>54</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>259</v>
+        <v>311</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>29</v>
@@ -6506,7 +6872,10 @@
         <v>104</v>
       </c>
       <c r="O58" s="3" t="s">
-        <v>260</v>
+        <v>312</v>
+      </c>
+      <c r="P58" s="8" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="59">
@@ -6517,7 +6886,7 @@
         <v>36</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>261</v>
+        <v>314</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>14</v>
@@ -6548,7 +6917,10 @@
         <v>10</v>
       </c>
       <c r="O59" s="3" t="s">
-        <v>262</v>
+        <v>315</v>
+      </c>
+      <c r="P59" s="8" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="60">
@@ -6559,7 +6931,7 @@
         <v>41</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>263</v>
+        <v>317</v>
       </c>
       <c r="D60" s="1" t="s">
         <v>14</v>
@@ -6593,7 +6965,10 @@
         <v>10</v>
       </c>
       <c r="O60" s="3" t="s">
-        <v>264</v>
+        <v>318</v>
+      </c>
+      <c r="P60" s="8" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="61">
@@ -6604,7 +6979,7 @@
         <v>36</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>265</v>
+        <v>320</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>14</v>
@@ -6634,7 +7009,10 @@
         <v>104</v>
       </c>
       <c r="O61" s="3" t="s">
-        <v>266</v>
+        <v>321</v>
+      </c>
+      <c r="P61" s="8" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="62">
@@ -6645,7 +7023,7 @@
         <v>31</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>267</v>
+        <v>323</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>32</v>
@@ -6676,6 +7054,9 @@
       </c>
       <c r="N62" s="3" t="s">
         <v>10</v>
+      </c>
+      <c r="P62" s="8" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="63">
@@ -6686,7 +7067,7 @@
         <v>24</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>268</v>
+        <v>325</v>
       </c>
       <c r="D63" s="1" t="s">
         <v>14</v>
@@ -6719,7 +7100,10 @@
         <v>10</v>
       </c>
       <c r="O63" s="8" t="s">
-        <v>269</v>
+        <v>326</v>
+      </c>
+      <c r="P63" s="8" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="64">
@@ -6730,7 +7114,7 @@
         <v>24</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>268</v>
+        <v>325</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>14</v>
@@ -6740,7 +7124,7 @@
       </c>
       <c r="F64" s="1"/>
       <c r="G64" s="1" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="H64" s="1" t="s">
         <v>17</v>
@@ -6761,7 +7145,10 @@
         <v>10</v>
       </c>
       <c r="O64" s="8" t="s">
-        <v>269</v>
+        <v>326</v>
+      </c>
+      <c r="P64" s="8" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="65">
@@ -6772,7 +7159,7 @@
         <v>98</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>270</v>
+        <v>329</v>
       </c>
       <c r="D65" s="1" t="s">
         <v>14</v>
@@ -6802,7 +7189,10 @@
         <v>10</v>
       </c>
       <c r="O65" s="3" t="s">
-        <v>271</v>
+        <v>330</v>
+      </c>
+      <c r="P65" s="8" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="66">
@@ -6813,7 +7203,7 @@
         <v>91</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>272</v>
+        <v>332</v>
       </c>
       <c r="D66" s="1" t="s">
         <v>14</v>
@@ -6844,7 +7234,10 @@
         <v>10</v>
       </c>
       <c r="O66" s="3" t="s">
-        <v>273</v>
+        <v>333</v>
+      </c>
+      <c r="P66" s="3" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="67">
@@ -6855,7 +7248,7 @@
         <v>37</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>274</v>
+        <v>335</v>
       </c>
       <c r="D67" s="1" t="s">
         <v>38</v>
@@ -6889,7 +7282,10 @@
         <v>10</v>
       </c>
       <c r="O67" s="3" t="s">
-        <v>275</v>
+        <v>336</v>
+      </c>
+      <c r="P67" s="3" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="68">
@@ -6900,7 +7296,7 @@
         <v>37</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>276</v>
+        <v>338</v>
       </c>
       <c r="D68" s="1" t="s">
         <v>38</v>
@@ -6931,7 +7327,10 @@
         <v>10</v>
       </c>
       <c r="O68" s="3" t="s">
-        <v>277</v>
+        <v>339</v>
+      </c>
+      <c r="P68" s="3" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="69">
@@ -6942,7 +7341,7 @@
         <v>94</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>229</v>
+        <v>262</v>
       </c>
       <c r="D69" s="1" t="s">
         <v>46</v>
@@ -6972,6 +7371,9 @@
       <c r="N69" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="P69" s="3" t="s">
+        <v>341</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="7">
@@ -6981,7 +7383,7 @@
         <v>58</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>229</v>
+        <v>262</v>
       </c>
       <c r="D70" s="1" t="s">
         <v>14</v>
@@ -6990,7 +7392,7 @@
         <v>35</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>278</v>
+        <v>342</v>
       </c>
       <c r="G70" s="1" t="s">
         <v>16</v>
@@ -7017,7 +7419,10 @@
         <v>10</v>
       </c>
       <c r="O70" s="3" t="s">
-        <v>279</v>
+        <v>343</v>
+      </c>
+      <c r="P70" s="3" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="71">
@@ -7028,7 +7433,7 @@
         <v>41</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>280</v>
+        <v>345</v>
       </c>
       <c r="D71" s="1" t="s">
         <v>43</v>
@@ -7064,7 +7469,10 @@
         <v>10</v>
       </c>
       <c r="O71" s="3" t="s">
-        <v>281</v>
+        <v>346</v>
+      </c>
+      <c r="P71" s="3" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="72">
@@ -7072,10 +7480,10 @@
         <v>46129.0</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>282</v>
+        <v>348</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>283</v>
+        <v>349</v>
       </c>
       <c r="D72" s="1" t="s">
         <v>88</v>
@@ -7085,7 +7493,7 @@
       </c>
       <c r="F72" s="1"/>
       <c r="G72" s="1" t="s">
-        <v>284</v>
+        <v>350</v>
       </c>
       <c r="H72" s="1" t="s">
         <v>17</v>
@@ -7106,7 +7514,10 @@
         <v>10</v>
       </c>
       <c r="O72" s="3" t="s">
-        <v>285</v>
+        <v>351</v>
+      </c>
+      <c r="P72" s="8" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="73">
@@ -9916,134 +10327,203 @@
   <hyperlinks>
     <hyperlink r:id="rId1" ref="N2"/>
     <hyperlink r:id="rId2" ref="O2"/>
-    <hyperlink r:id="rId3" ref="N3"/>
-    <hyperlink r:id="rId4" ref="O3"/>
-    <hyperlink r:id="rId5" ref="N4"/>
-    <hyperlink r:id="rId6" ref="O4"/>
-    <hyperlink r:id="rId7" ref="N5"/>
-    <hyperlink r:id="rId8" ref="O5"/>
-    <hyperlink r:id="rId9" ref="N6"/>
-    <hyperlink r:id="rId10" ref="O6"/>
-    <hyperlink r:id="rId11" ref="N7"/>
-    <hyperlink r:id="rId12" ref="O7"/>
-    <hyperlink r:id="rId13" ref="N8"/>
-    <hyperlink r:id="rId14" ref="O8"/>
-    <hyperlink r:id="rId15" ref="N9"/>
-    <hyperlink r:id="rId16" ref="O9"/>
-    <hyperlink r:id="rId17" ref="N10"/>
-    <hyperlink r:id="rId18" ref="O10"/>
-    <hyperlink r:id="rId19" ref="N11"/>
-    <hyperlink r:id="rId20" ref="O11"/>
-    <hyperlink r:id="rId21" ref="N12"/>
-    <hyperlink r:id="rId22" ref="O12"/>
-    <hyperlink r:id="rId23" ref="N13"/>
-    <hyperlink r:id="rId24" ref="O13"/>
-    <hyperlink r:id="rId25" ref="N14"/>
-    <hyperlink r:id="rId26" ref="O14"/>
-    <hyperlink r:id="rId27" ref="N15"/>
-    <hyperlink r:id="rId28" ref="O15"/>
-    <hyperlink r:id="rId29" ref="N16"/>
-    <hyperlink r:id="rId30" ref="O16"/>
-    <hyperlink r:id="rId31" ref="O17"/>
-    <hyperlink r:id="rId32" ref="N18"/>
-    <hyperlink r:id="rId33" ref="O18"/>
-    <hyperlink r:id="rId34" ref="N19"/>
-    <hyperlink r:id="rId35" ref="O19"/>
-    <hyperlink r:id="rId36" ref="N20"/>
-    <hyperlink r:id="rId37" ref="O20"/>
-    <hyperlink r:id="rId38" ref="N21"/>
-    <hyperlink r:id="rId39" ref="N22"/>
-    <hyperlink r:id="rId40" ref="O22"/>
-    <hyperlink r:id="rId41" ref="N23"/>
-    <hyperlink r:id="rId42" ref="O23"/>
-    <hyperlink r:id="rId43" ref="N24"/>
-    <hyperlink r:id="rId44" ref="O24"/>
-    <hyperlink r:id="rId45" ref="N25"/>
-    <hyperlink r:id="rId46" ref="N26"/>
-    <hyperlink r:id="rId47" ref="O26"/>
-    <hyperlink r:id="rId48" ref="N27"/>
-    <hyperlink r:id="rId49" ref="O27"/>
-    <hyperlink r:id="rId50" ref="N28"/>
-    <hyperlink r:id="rId51" ref="N29"/>
-    <hyperlink r:id="rId52" ref="O29"/>
-    <hyperlink r:id="rId53" ref="N30"/>
-    <hyperlink r:id="rId54" ref="N31"/>
-    <hyperlink r:id="rId55" ref="O31"/>
-    <hyperlink r:id="rId56" ref="N32"/>
-    <hyperlink r:id="rId57" ref="O32"/>
-    <hyperlink r:id="rId58" ref="N33"/>
-    <hyperlink r:id="rId59" ref="O33"/>
-    <hyperlink r:id="rId60" ref="N34"/>
-    <hyperlink r:id="rId61" ref="O34"/>
-    <hyperlink r:id="rId62" ref="N35"/>
-    <hyperlink r:id="rId63" ref="N36"/>
-    <hyperlink r:id="rId64" ref="O36"/>
-    <hyperlink r:id="rId65" ref="N37"/>
-    <hyperlink r:id="rId66" ref="N38"/>
-    <hyperlink r:id="rId67" ref="N39"/>
-    <hyperlink r:id="rId68" ref="O39"/>
-    <hyperlink r:id="rId69" ref="N40"/>
-    <hyperlink r:id="rId70" ref="O40"/>
-    <hyperlink r:id="rId71" ref="N41"/>
-    <hyperlink r:id="rId72" ref="O41"/>
-    <hyperlink r:id="rId73" ref="N42"/>
-    <hyperlink r:id="rId74" ref="O42"/>
-    <hyperlink r:id="rId75" ref="N43"/>
-    <hyperlink r:id="rId76" ref="O43"/>
-    <hyperlink r:id="rId77" ref="N44"/>
-    <hyperlink r:id="rId78" ref="O44"/>
-    <hyperlink r:id="rId79" ref="N45"/>
-    <hyperlink r:id="rId80" ref="O45"/>
-    <hyperlink r:id="rId81" ref="N46"/>
-    <hyperlink r:id="rId82" ref="O46"/>
-    <hyperlink r:id="rId83" ref="N47"/>
-    <hyperlink r:id="rId84" ref="O47"/>
-    <hyperlink r:id="rId85" ref="N48"/>
-    <hyperlink r:id="rId86" ref="N49"/>
-    <hyperlink r:id="rId87" ref="O49"/>
-    <hyperlink r:id="rId88" ref="N50"/>
-    <hyperlink r:id="rId89" ref="O50"/>
-    <hyperlink r:id="rId90" ref="N51"/>
-    <hyperlink r:id="rId91" ref="O51"/>
-    <hyperlink r:id="rId92" ref="N52"/>
-    <hyperlink r:id="rId93" ref="O52"/>
-    <hyperlink r:id="rId94" ref="N53"/>
-    <hyperlink r:id="rId95" ref="O53"/>
-    <hyperlink r:id="rId96" ref="N54"/>
-    <hyperlink r:id="rId97" ref="O54"/>
-    <hyperlink r:id="rId98" ref="N55"/>
-    <hyperlink r:id="rId99" ref="O55"/>
-    <hyperlink r:id="rId100" ref="N56"/>
-    <hyperlink r:id="rId101" ref="O56"/>
-    <hyperlink r:id="rId102" ref="N57"/>
-    <hyperlink r:id="rId103" ref="O57"/>
-    <hyperlink r:id="rId104" ref="O58"/>
-    <hyperlink r:id="rId105" ref="N59"/>
-    <hyperlink r:id="rId106" ref="O59"/>
-    <hyperlink r:id="rId107" ref="N60"/>
-    <hyperlink r:id="rId108" ref="O60"/>
-    <hyperlink r:id="rId109" ref="O61"/>
-    <hyperlink r:id="rId110" ref="N62"/>
-    <hyperlink r:id="rId111" ref="N63"/>
-    <hyperlink r:id="rId112" ref="O63"/>
-    <hyperlink r:id="rId113" ref="N64"/>
-    <hyperlink r:id="rId114" ref="O64"/>
-    <hyperlink r:id="rId115" ref="N65"/>
-    <hyperlink r:id="rId116" ref="O65"/>
-    <hyperlink r:id="rId117" ref="N66"/>
-    <hyperlink r:id="rId118" ref="O66"/>
-    <hyperlink r:id="rId119" ref="N67"/>
-    <hyperlink r:id="rId120" ref="O67"/>
-    <hyperlink r:id="rId121" ref="N68"/>
-    <hyperlink r:id="rId122" ref="O68"/>
-    <hyperlink r:id="rId123" ref="N69"/>
-    <hyperlink r:id="rId124" ref="N70"/>
-    <hyperlink r:id="rId125" ref="O70"/>
-    <hyperlink r:id="rId126" ref="N71"/>
-    <hyperlink r:id="rId127" ref="O71"/>
-    <hyperlink r:id="rId128" ref="N72"/>
-    <hyperlink r:id="rId129" ref="O72"/>
+    <hyperlink r:id="rId3" ref="P2"/>
+    <hyperlink r:id="rId4" ref="N3"/>
+    <hyperlink r:id="rId5" ref="O3"/>
+    <hyperlink r:id="rId6" ref="P3"/>
+    <hyperlink r:id="rId7" ref="N4"/>
+    <hyperlink r:id="rId8" ref="O4"/>
+    <hyperlink r:id="rId9" ref="P4"/>
+    <hyperlink r:id="rId10" ref="N5"/>
+    <hyperlink r:id="rId11" ref="O5"/>
+    <hyperlink r:id="rId12" ref="P5"/>
+    <hyperlink r:id="rId13" ref="N6"/>
+    <hyperlink r:id="rId14" ref="O6"/>
+    <hyperlink r:id="rId15" ref="P6"/>
+    <hyperlink r:id="rId16" ref="N7"/>
+    <hyperlink r:id="rId17" ref="O7"/>
+    <hyperlink r:id="rId18" ref="P7"/>
+    <hyperlink r:id="rId19" ref="N8"/>
+    <hyperlink r:id="rId20" ref="O8"/>
+    <hyperlink r:id="rId21" ref="P8"/>
+    <hyperlink r:id="rId22" ref="N9"/>
+    <hyperlink r:id="rId23" ref="O9"/>
+    <hyperlink r:id="rId24" ref="P9"/>
+    <hyperlink r:id="rId25" ref="N10"/>
+    <hyperlink r:id="rId26" ref="O10"/>
+    <hyperlink r:id="rId27" ref="P10"/>
+    <hyperlink r:id="rId28" ref="N11"/>
+    <hyperlink r:id="rId29" ref="O11"/>
+    <hyperlink r:id="rId30" ref="P11"/>
+    <hyperlink r:id="rId31" ref="N12"/>
+    <hyperlink r:id="rId32" ref="O12"/>
+    <hyperlink r:id="rId33" ref="P12"/>
+    <hyperlink r:id="rId34" ref="N13"/>
+    <hyperlink r:id="rId35" ref="O13"/>
+    <hyperlink r:id="rId36" ref="P13"/>
+    <hyperlink r:id="rId37" ref="N14"/>
+    <hyperlink r:id="rId38" ref="O14"/>
+    <hyperlink r:id="rId39" ref="P14"/>
+    <hyperlink r:id="rId40" ref="N15"/>
+    <hyperlink r:id="rId41" ref="O15"/>
+    <hyperlink r:id="rId42" ref="P15"/>
+    <hyperlink r:id="rId43" ref="N16"/>
+    <hyperlink r:id="rId44" ref="O16"/>
+    <hyperlink r:id="rId45" ref="P16"/>
+    <hyperlink r:id="rId46" ref="O17"/>
+    <hyperlink r:id="rId47" ref="P17"/>
+    <hyperlink r:id="rId48" ref="N18"/>
+    <hyperlink r:id="rId49" ref="O18"/>
+    <hyperlink r:id="rId50" ref="P18"/>
+    <hyperlink r:id="rId51" ref="N19"/>
+    <hyperlink r:id="rId52" ref="O19"/>
+    <hyperlink r:id="rId53" ref="P19"/>
+    <hyperlink r:id="rId54" ref="N20"/>
+    <hyperlink r:id="rId55" ref="O20"/>
+    <hyperlink r:id="rId56" ref="P20"/>
+    <hyperlink r:id="rId57" ref="N21"/>
+    <hyperlink r:id="rId58" ref="P21"/>
+    <hyperlink r:id="rId59" ref="N22"/>
+    <hyperlink r:id="rId60" ref="O22"/>
+    <hyperlink r:id="rId61" ref="P22"/>
+    <hyperlink r:id="rId62" ref="N23"/>
+    <hyperlink r:id="rId63" ref="O23"/>
+    <hyperlink r:id="rId64" ref="P23"/>
+    <hyperlink r:id="rId65" ref="N24"/>
+    <hyperlink r:id="rId66" ref="O24"/>
+    <hyperlink r:id="rId67" ref="P24"/>
+    <hyperlink r:id="rId68" ref="N25"/>
+    <hyperlink r:id="rId69" ref="P25"/>
+    <hyperlink r:id="rId70" ref="N26"/>
+    <hyperlink r:id="rId71" ref="O26"/>
+    <hyperlink r:id="rId72" ref="P26"/>
+    <hyperlink r:id="rId73" ref="N27"/>
+    <hyperlink r:id="rId74" ref="O27"/>
+    <hyperlink r:id="rId75" ref="P27"/>
+    <hyperlink r:id="rId76" ref="N28"/>
+    <hyperlink r:id="rId77" ref="N29"/>
+    <hyperlink r:id="rId78" ref="O29"/>
+    <hyperlink r:id="rId79" ref="P29"/>
+    <hyperlink r:id="rId80" ref="N30"/>
+    <hyperlink r:id="rId81" ref="P30"/>
+    <hyperlink r:id="rId82" ref="N31"/>
+    <hyperlink r:id="rId83" ref="O31"/>
+    <hyperlink r:id="rId84" ref="P31"/>
+    <hyperlink r:id="rId85" ref="N32"/>
+    <hyperlink r:id="rId86" ref="O32"/>
+    <hyperlink r:id="rId87" ref="P32"/>
+    <hyperlink r:id="rId88" ref="N33"/>
+    <hyperlink r:id="rId89" ref="O33"/>
+    <hyperlink r:id="rId90" ref="P33"/>
+    <hyperlink r:id="rId91" ref="N34"/>
+    <hyperlink r:id="rId92" ref="O34"/>
+    <hyperlink r:id="rId93" ref="P34"/>
+    <hyperlink r:id="rId94" ref="N35"/>
+    <hyperlink r:id="rId95" ref="N36"/>
+    <hyperlink r:id="rId96" ref="O36"/>
+    <hyperlink r:id="rId97" ref="P36"/>
+    <hyperlink r:id="rId98" ref="N37"/>
+    <hyperlink r:id="rId99" ref="P37"/>
+    <hyperlink r:id="rId100" ref="N38"/>
+    <hyperlink r:id="rId101" ref="P38"/>
+    <hyperlink r:id="rId102" ref="N39"/>
+    <hyperlink r:id="rId103" ref="O39"/>
+    <hyperlink r:id="rId104" ref="P39"/>
+    <hyperlink r:id="rId105" ref="N40"/>
+    <hyperlink r:id="rId106" ref="O40"/>
+    <hyperlink r:id="rId107" ref="P40"/>
+    <hyperlink r:id="rId108" ref="N41"/>
+    <hyperlink r:id="rId109" ref="O41"/>
+    <hyperlink r:id="rId110" ref="P41"/>
+    <hyperlink r:id="rId111" ref="N42"/>
+    <hyperlink r:id="rId112" ref="O42"/>
+    <hyperlink r:id="rId113" ref="P42"/>
+    <hyperlink r:id="rId114" ref="N43"/>
+    <hyperlink r:id="rId115" ref="O43"/>
+    <hyperlink r:id="rId116" ref="P43"/>
+    <hyperlink r:id="rId117" ref="N44"/>
+    <hyperlink r:id="rId118" ref="O44"/>
+    <hyperlink r:id="rId119" ref="P44"/>
+    <hyperlink r:id="rId120" ref="N45"/>
+    <hyperlink r:id="rId121" ref="O45"/>
+    <hyperlink r:id="rId122" ref="P45"/>
+    <hyperlink r:id="rId123" ref="N46"/>
+    <hyperlink r:id="rId124" ref="O46"/>
+    <hyperlink r:id="rId125" ref="P46"/>
+    <hyperlink r:id="rId126" ref="N47"/>
+    <hyperlink r:id="rId127" ref="O47"/>
+    <hyperlink r:id="rId128" ref="P47"/>
+    <hyperlink r:id="rId129" ref="N48"/>
+    <hyperlink r:id="rId130" ref="P48"/>
+    <hyperlink r:id="rId131" ref="N49"/>
+    <hyperlink r:id="rId132" ref="O49"/>
+    <hyperlink r:id="rId133" ref="P49"/>
+    <hyperlink r:id="rId134" ref="N50"/>
+    <hyperlink r:id="rId135" ref="O50"/>
+    <hyperlink r:id="rId136" ref="P50"/>
+    <hyperlink r:id="rId137" ref="N51"/>
+    <hyperlink r:id="rId138" ref="O51"/>
+    <hyperlink r:id="rId139" ref="P51"/>
+    <hyperlink r:id="rId140" ref="N52"/>
+    <hyperlink r:id="rId141" ref="O52"/>
+    <hyperlink r:id="rId142" ref="P52"/>
+    <hyperlink r:id="rId143" ref="N53"/>
+    <hyperlink r:id="rId144" ref="O53"/>
+    <hyperlink r:id="rId145" ref="P53"/>
+    <hyperlink r:id="rId146" ref="N54"/>
+    <hyperlink r:id="rId147" ref="O54"/>
+    <hyperlink r:id="rId148" ref="P54"/>
+    <hyperlink r:id="rId149" ref="N55"/>
+    <hyperlink r:id="rId150" ref="O55"/>
+    <hyperlink r:id="rId151" ref="P55"/>
+    <hyperlink r:id="rId152" ref="N56"/>
+    <hyperlink r:id="rId153" ref="O56"/>
+    <hyperlink r:id="rId154" ref="P56"/>
+    <hyperlink r:id="rId155" ref="N57"/>
+    <hyperlink r:id="rId156" ref="O57"/>
+    <hyperlink r:id="rId157" ref="P57"/>
+    <hyperlink r:id="rId158" ref="O58"/>
+    <hyperlink r:id="rId159" ref="P58"/>
+    <hyperlink r:id="rId160" ref="N59"/>
+    <hyperlink r:id="rId161" ref="O59"/>
+    <hyperlink r:id="rId162" ref="P59"/>
+    <hyperlink r:id="rId163" ref="N60"/>
+    <hyperlink r:id="rId164" ref="O60"/>
+    <hyperlink r:id="rId165" ref="P60"/>
+    <hyperlink r:id="rId166" ref="O61"/>
+    <hyperlink r:id="rId167" ref="P61"/>
+    <hyperlink r:id="rId168" ref="N62"/>
+    <hyperlink r:id="rId169" ref="P62"/>
+    <hyperlink r:id="rId170" ref="N63"/>
+    <hyperlink r:id="rId171" ref="O63"/>
+    <hyperlink r:id="rId172" ref="P63"/>
+    <hyperlink r:id="rId173" ref="N64"/>
+    <hyperlink r:id="rId174" ref="O64"/>
+    <hyperlink r:id="rId175" ref="P64"/>
+    <hyperlink r:id="rId176" ref="N65"/>
+    <hyperlink r:id="rId177" ref="O65"/>
+    <hyperlink r:id="rId178" ref="P65"/>
+    <hyperlink r:id="rId179" ref="N66"/>
+    <hyperlink r:id="rId180" ref="O66"/>
+    <hyperlink r:id="rId181" ref="P66"/>
+    <hyperlink r:id="rId182" ref="N67"/>
+    <hyperlink r:id="rId183" ref="O67"/>
+    <hyperlink r:id="rId184" ref="P67"/>
+    <hyperlink r:id="rId185" ref="N68"/>
+    <hyperlink r:id="rId186" ref="O68"/>
+    <hyperlink r:id="rId187" ref="P68"/>
+    <hyperlink r:id="rId188" ref="N69"/>
+    <hyperlink r:id="rId189" ref="P69"/>
+    <hyperlink r:id="rId190" ref="N70"/>
+    <hyperlink r:id="rId191" ref="O70"/>
+    <hyperlink r:id="rId192" ref="P70"/>
+    <hyperlink r:id="rId193" ref="N71"/>
+    <hyperlink r:id="rId194" ref="O71"/>
+    <hyperlink r:id="rId195" ref="P71"/>
+    <hyperlink r:id="rId196" ref="N72"/>
+    <hyperlink r:id="rId197" ref="O72"/>
+    <hyperlink r:id="rId198" ref="P72"/>
   </hyperlinks>
-  <drawing r:id="rId130"/>
+  <drawing r:id="rId199"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix System of a Down date 8/27 → 8/28
</commit_message>
<xml_diff>
--- a/Poster Collection.xlsx
+++ b/Poster Collection.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="325">
   <si>
     <t>Date</t>
   </si>
@@ -469,6 +469,9 @@
   </si>
   <si>
     <t>https://expressobeans.com/public/detail.php/301920</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1qhtkrXebdTxDmKdGWpDHEcFOrOEQbjaW/view?usp=drive_link</t>
   </si>
   <si>
     <t>KISS</t>
@@ -2598,7 +2601,7 @@
         <v>151</v>
       </c>
       <c r="P29" s="4" t="s">
-        <v>109</v>
+        <v>152</v>
       </c>
     </row>
     <row r="30">
@@ -2606,10 +2609,10 @@
         <v>43561.0</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>39</v>
@@ -2645,13 +2648,13 @@
         <v>43595.0</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>19</v>
@@ -2679,10 +2682,10 @@
         <v>26</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P31" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="32">
@@ -2693,7 +2696,7 @@
         <v>110</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>79</v>
@@ -2703,7 +2706,7 @@
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>22</v>
@@ -2718,7 +2721,7 @@
         <v>24</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="M32" s="2">
         <v>23.0</v>
@@ -2727,7 +2730,7 @@
         <v>26</v>
       </c>
       <c r="P32" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33">
@@ -2748,7 +2751,7 @@
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>22</v>
@@ -2772,10 +2775,10 @@
         <v>26</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="P33" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="34">
@@ -2786,7 +2789,7 @@
         <v>84</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>39</v>
@@ -2796,7 +2799,7 @@
       </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>22</v>
@@ -2820,10 +2823,10 @@
         <v>26</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P34" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35">
@@ -2834,17 +2837,17 @@
         <v>84</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F35" s="2"/>
       <c r="G35" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>22</v>
@@ -2859,7 +2862,7 @@
         <v>23</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="M35" s="2" t="s">
         <v>25</v>
@@ -2868,10 +2871,10 @@
         <v>26</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P35" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="36">
@@ -2882,17 +2885,17 @@
         <v>84</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H36" s="2" t="s">
         <v>22</v>
@@ -2913,10 +2916,10 @@
         <v>26</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="P36" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="37">
@@ -2924,13 +2927,13 @@
         <v>43869.0</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>32</v>
@@ -2952,7 +2955,7 @@
         <v>24</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M37" s="2">
         <v>31.0</v>
@@ -2966,10 +2969,10 @@
         <v>44450.0</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>39</v>
@@ -2979,7 +2982,7 @@
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>34</v>
@@ -3000,10 +3003,10 @@
         <v>26</v>
       </c>
       <c r="O38" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="P38" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="39">
@@ -3014,7 +3017,7 @@
         <v>110</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>39</v>
@@ -3024,7 +3027,7 @@
       </c>
       <c r="F39" s="2"/>
       <c r="G39" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>22</v>
@@ -3045,7 +3048,7 @@
         <v>26</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="40">
@@ -3053,19 +3056,19 @@
         <v>44511.0</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>33</v>
@@ -3089,7 +3092,7 @@
         <v>26</v>
       </c>
       <c r="P40" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="41">
@@ -3097,10 +3100,10 @@
         <v>44519.0</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>39</v>
@@ -3110,7 +3113,7 @@
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>34</v>
@@ -3131,10 +3134,10 @@
         <v>26</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="P41" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="42">
@@ -3145,17 +3148,17 @@
         <v>84</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>22</v>
@@ -3170,7 +3173,7 @@
         <v>24</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>25</v>
@@ -3179,10 +3182,10 @@
         <v>26</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="43">
@@ -3193,10 +3196,10 @@
         <v>84</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>32</v>
@@ -3224,10 +3227,10 @@
         <v>26</v>
       </c>
       <c r="O43" s="4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="44">
@@ -3238,7 +3241,7 @@
         <v>37</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>39</v>
@@ -3248,7 +3251,7 @@
       </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>22</v>
@@ -3269,10 +3272,10 @@
         <v>26</v>
       </c>
       <c r="O44" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="45">
@@ -3283,7 +3286,7 @@
         <v>37</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>39</v>
@@ -3293,7 +3296,7 @@
       </c>
       <c r="F45" s="2"/>
       <c r="G45" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>22</v>
@@ -3314,10 +3317,10 @@
         <v>26</v>
       </c>
       <c r="O45" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="P45" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="46">
@@ -3328,19 +3331,19 @@
         <v>77</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>22</v>
@@ -3361,10 +3364,10 @@
         <v>26</v>
       </c>
       <c r="O46" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="P46" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="47">
@@ -3372,10 +3375,10 @@
         <v>44773.0</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>39</v>
@@ -3406,10 +3409,10 @@
         <v>26</v>
       </c>
       <c r="O47" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="P47" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="48">
@@ -3417,13 +3420,13 @@
         <v>44804.0</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>32</v>
@@ -3451,10 +3454,10 @@
         <v>26</v>
       </c>
       <c r="O48" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="P48" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="49">
@@ -3475,7 +3478,7 @@
       </c>
       <c r="F49" s="2"/>
       <c r="G49" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H49" s="2" t="s">
         <v>22</v>
@@ -3496,10 +3499,10 @@
         <v>26</v>
       </c>
       <c r="O49" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="P49" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="50">
@@ -3507,19 +3510,19 @@
         <v>45064.0</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>117</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>33</v>
@@ -3543,7 +3546,7 @@
         <v>26</v>
       </c>
       <c r="P50" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="51">
@@ -3554,17 +3557,17 @@
         <v>84</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F51" s="2"/>
       <c r="G51" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H51" s="2" t="s">
         <v>22</v>
@@ -3585,10 +3588,10 @@
         <v>26</v>
       </c>
       <c r="O51" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="P51" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="52">
@@ -3599,17 +3602,17 @@
         <v>92</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>22</v>
@@ -3624,7 +3627,7 @@
         <v>24</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M52" s="2">
         <v>12.0</v>
@@ -3633,10 +3636,10 @@
         <v>26</v>
       </c>
       <c r="O52" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="P52" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="53">
@@ -3647,17 +3650,17 @@
         <v>92</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="H53" s="2" t="s">
         <v>22</v>
@@ -3672,7 +3675,7 @@
         <v>23</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="M53" s="2">
         <v>13.0</v>
@@ -3681,10 +3684,10 @@
         <v>26</v>
       </c>
       <c r="O53" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="P53" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="54">
@@ -3692,13 +3695,13 @@
         <v>45213.0</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>32</v>
@@ -3727,10 +3730,10 @@
         <v>26</v>
       </c>
       <c r="O54" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="P54" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="55">
@@ -3738,10 +3741,10 @@
         <v>45228.0</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>39</v>
@@ -3750,7 +3753,7 @@
         <v>32</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>33</v>
@@ -3774,10 +3777,10 @@
         <v>26</v>
       </c>
       <c r="O55" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="P55" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="56">
@@ -3785,10 +3788,10 @@
         <v>45228.0</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>39</v>
@@ -3798,7 +3801,7 @@
       </c>
       <c r="F56" s="2"/>
       <c r="G56" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>34</v>
@@ -3819,10 +3822,10 @@
         <v>26</v>
       </c>
       <c r="O56" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="P56" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="57">
@@ -3830,10 +3833,10 @@
         <v>45239.0</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>39</v>
@@ -3864,10 +3867,10 @@
         <v>26</v>
       </c>
       <c r="O57" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="P57" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="58">
@@ -3878,7 +3881,7 @@
         <v>84</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>79</v>
@@ -3888,7 +3891,7 @@
       </c>
       <c r="F58" s="2"/>
       <c r="G58" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>22</v>
@@ -3909,10 +3912,10 @@
         <v>26</v>
       </c>
       <c r="O58" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="P58" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="59">
@@ -3923,7 +3926,7 @@
         <v>84</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>79</v>
@@ -3933,7 +3936,7 @@
       </c>
       <c r="F59" s="2"/>
       <c r="G59" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>22</v>
@@ -3954,10 +3957,10 @@
         <v>26</v>
       </c>
       <c r="O59" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="P59" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="60">
@@ -3968,10 +3971,10 @@
         <v>84</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>32</v>
@@ -3989,16 +3992,16 @@
         <v>24</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="M60" s="2" t="s">
         <v>25</v>
       </c>
       <c r="O60" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="P60" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="61">
@@ -4006,10 +4009,10 @@
         <v>45389.0</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>39</v>
@@ -4040,10 +4043,10 @@
         <v>26</v>
       </c>
       <c r="O61" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P61" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="62">
@@ -4051,10 +4054,10 @@
         <v>45389.0</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>39</v>
@@ -4079,7 +4082,7 @@
         <v>24</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="M62" s="2">
         <v>9.0</v>
@@ -4088,10 +4091,10 @@
         <v>26</v>
       </c>
       <c r="O62" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="P62" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="63">
@@ -4099,10 +4102,10 @@
         <v>45389.0</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>39</v>
@@ -4111,7 +4114,7 @@
         <v>32</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>22</v>
@@ -4126,16 +4129,16 @@
         <v>24</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="M63" s="2" t="s">
         <v>25</v>
       </c>
       <c r="O63" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="P63" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="64">
@@ -4143,10 +4146,10 @@
         <v>45428.0</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>126</v>
@@ -4155,7 +4158,7 @@
         <v>32</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>33</v>
@@ -4179,7 +4182,7 @@
         <v>26</v>
       </c>
       <c r="P64" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="65">
@@ -4187,10 +4190,10 @@
         <v>45469.0</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>39</v>
@@ -4199,10 +4202,10 @@
         <v>19</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H65" s="2" t="s">
         <v>22</v>
@@ -4223,10 +4226,10 @@
         <v>26</v>
       </c>
       <c r="O65" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P65" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="66">
@@ -4234,10 +4237,10 @@
         <v>45469.0</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>39</v>
@@ -4268,10 +4271,10 @@
         <v>26</v>
       </c>
       <c r="O66" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P66" s="4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="67">
@@ -4279,10 +4282,10 @@
         <v>45783.0</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>39</v>
@@ -4291,7 +4294,7 @@
         <v>19</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H67" s="2" t="s">
         <v>22</v>
@@ -4312,10 +4315,10 @@
         <v>26</v>
       </c>
       <c r="O67" s="3" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="P67" s="4" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="68">
@@ -4357,10 +4360,10 @@
         <v>26</v>
       </c>
       <c r="O68" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="P68" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="69">
@@ -4371,7 +4374,7 @@
         <v>92</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>79</v>
@@ -4381,7 +4384,7 @@
       </c>
       <c r="F69" s="2"/>
       <c r="G69" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>22</v>
@@ -4396,7 +4399,7 @@
         <v>24</v>
       </c>
       <c r="L69" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="M69" s="2">
         <v>8.0</v>
@@ -4405,10 +4408,10 @@
         <v>26</v>
       </c>
       <c r="O69" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="P69" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="70">
@@ -4419,7 +4422,7 @@
         <v>92</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>79</v>
@@ -4429,7 +4432,7 @@
       </c>
       <c r="F70" s="2"/>
       <c r="G70" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>22</v>
@@ -4450,24 +4453,24 @@
         <v>26</v>
       </c>
       <c r="O70" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="P70" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1">
-        <v>45896.0</v>
+        <v>45897.0</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>32</v>
@@ -4495,7 +4498,7 @@
         <v>26</v>
       </c>
       <c r="P71" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="72">
@@ -4506,7 +4509,7 @@
         <v>37</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>39</v>
@@ -4515,7 +4518,7 @@
         <v>32</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G72" s="2" t="s">
         <v>33</v>
@@ -4533,7 +4536,7 @@
         <v>24</v>
       </c>
       <c r="L72" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="M72" s="2">
         <v>35.0</v>
@@ -4542,10 +4545,10 @@
         <v>26</v>
       </c>
       <c r="O72" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="P72" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="73">
@@ -4556,19 +4559,19 @@
         <v>77</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>22</v>
@@ -4583,7 +4586,7 @@
         <v>24</v>
       </c>
       <c r="L73" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="M73" s="2">
         <v>11.0</v>
@@ -4592,10 +4595,10 @@
         <v>26</v>
       </c>
       <c r="O73" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="P73" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="74">
@@ -4603,20 +4606,20 @@
         <v>46129.0</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F74" s="2"/>
       <c r="G74" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="H74" s="2" t="s">
         <v>22</v>
@@ -4635,10 +4638,10 @@
       </c>
       <c r="N74" s="9"/>
       <c r="O74" s="3" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="P74" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="75">

</xml_diff>